<commit_message>
Données API-only, titres v4, méthodo site, script de vérification
</commit_message>
<xml_diff>
--- a/charts/output/terra_nova_migrations_dataviz.xlsx
+++ b/charts/output/terra_nova_migrations_dataviz.xlsx
@@ -1077,7 +1077,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2.2</t>
+          <t>4.2</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1104,7 +1104,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>4.3</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1131,7 +1131,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2.2</t>
+          <t>2.8</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2.2</t>
+          <t>2.8</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1168,12 +1168,12 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>4.1</t>
+          <t>4.3</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>11.8</t>
+          <t>12.8</t>
         </is>
       </c>
     </row>
@@ -1405,37 +1405,37 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>France (entière) (2024)</t>
+          <t>Suède (2024)</t>
         </is>
       </c>
       <c r="C5" t="n">
         <v>2024</v>
       </c>
       <c r="D5" t="n">
-        <v>2.2</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>FR</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Suède (2024)</t>
+          <t>France (entière) (2024)</t>
         </is>
       </c>
       <c r="C6" t="n">
         <v>2024</v>
       </c>
       <c r="D6" t="n">
-        <v>2.7</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="7">
@@ -1453,7 +1453,7 @@
         <v>2024</v>
       </c>
       <c r="D7" t="n">
-        <v>4.1</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="8">
@@ -1525,7 +1525,7 @@
         <v>2024</v>
       </c>
       <c r="D11" t="n">
-        <v>11.8</v>
+        <v>12.8</v>
       </c>
     </row>
     <row r="14">
@@ -1756,7 +1756,7 @@
         <v>2024</v>
       </c>
       <c r="D3" t="n">
-        <v>2.2</v>
+        <v>2.8</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -1784,7 +1784,7 @@
         <v>2024</v>
       </c>
       <c r="D4" t="n">
-        <v>4.1</v>
+        <v>4.3</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -2224,7 +2224,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2.2</t>
+          <t>4.2</t>
         </is>
       </c>
       <c r="C20" t="inlineStr"/>
@@ -2242,7 +2242,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4.3</t>
         </is>
       </c>
       <c r="C21" t="inlineStr"/>
@@ -2260,7 +2260,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2.2</t>
+          <t>2.8</t>
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
@@ -2278,7 +2278,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2.2</t>
+          <t>2.8</t>
         </is>
       </c>
       <c r="C23" t="inlineStr"/>
@@ -2659,7 +2659,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2.2</t>
+          <t>4.2</t>
         </is>
       </c>
       <c r="C20" t="inlineStr"/>
@@ -2677,7 +2677,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4.3</t>
         </is>
       </c>
       <c r="C21" t="inlineStr"/>
@@ -2695,7 +2695,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2.2</t>
+          <t>2.8</t>
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
@@ -2713,13 +2713,13 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2.2</t>
+          <t>2.8</t>
         </is>
       </c>
       <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr">
         <is>
-          <t>4.1</t>
+          <t>4.3</t>
         </is>
       </c>
     </row>
@@ -3094,7 +3094,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2.2</t>
+          <t>4.2</t>
         </is>
       </c>
       <c r="C20" t="inlineStr"/>
@@ -3112,7 +3112,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4.3</t>
         </is>
       </c>
       <c r="C21" t="inlineStr"/>
@@ -3130,7 +3130,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2.2</t>
+          <t>2.8</t>
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
@@ -3148,7 +3148,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2.2</t>
+          <t>2.8</t>
         </is>
       </c>
       <c r="C23" t="inlineStr"/>
@@ -3444,7 +3444,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2.2</t>
+          <t>4.2</t>
         </is>
       </c>
       <c r="C19" t="inlineStr"/>
@@ -3457,7 +3457,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4.3</t>
         </is>
       </c>
       <c r="C20" t="inlineStr"/>
@@ -3470,7 +3470,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2.2</t>
+          <t>2.8</t>
         </is>
       </c>
       <c r="C21" t="inlineStr"/>
@@ -3483,7 +3483,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2.2</t>
+          <t>2.8</t>
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
@@ -4217,7 +4217,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2.2</t>
+          <t>4.2</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -4259,7 +4259,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4.3</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -4301,7 +4301,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2.2</t>
+          <t>2.8</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -4343,7 +4343,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2.2</t>
+          <t>2.8</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -4353,7 +4353,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>11.8</t>
+          <t>12.8</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -4368,7 +4368,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>4.1</t>
+          <t>4.3</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -5366,7 +5366,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>7.2</t>
+          <t>5.9</t>
         </is>
       </c>
     </row>
@@ -5400,7 +5400,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>10.6</t>
+          <t>13.9</t>
         </is>
       </c>
     </row>
@@ -5485,7 +5485,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>6.4</t>
+          <t>5.2</t>
         </is>
       </c>
     </row>
@@ -5502,7 +5502,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>11.8</t>
+          <t>12.8</t>
         </is>
       </c>
     </row>
@@ -5536,7 +5536,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2.2</t>
+          <t>2.8</t>
         </is>
       </c>
     </row>
@@ -5587,7 +5587,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>12.8</t>
+          <t>13.1</t>
         </is>
       </c>
     </row>
@@ -5604,7 +5604,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>4.1</t>
+          <t>4.3</t>
         </is>
       </c>
     </row>
@@ -5655,7 +5655,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>-2.5</t>
+          <t>-2.3</t>
         </is>
       </c>
     </row>
@@ -5740,7 +5740,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>3.7</t>
+          <t>4.0</t>
         </is>
       </c>
     </row>
@@ -6163,7 +6163,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>0.8</t>
         </is>
       </c>
     </row>
@@ -6175,7 +6175,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>18</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -6283,7 +6283,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>16</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -6293,7 +6293,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2.2</t>
+          <t>4.2</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -6310,7 +6310,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>21</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -6320,7 +6320,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>4.3</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -6337,7 +6337,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>22</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -6347,7 +6347,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2.2</t>
+          <t>2.8</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -6364,7 +6364,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>21</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -6374,7 +6374,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2.2</t>
+          <t>2.8</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -9363,7 +9363,7 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>2.2</t>
+          <t>4.2</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
@@ -9373,7 +9373,7 @@
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>0.6967</t>
+          <t>0.3649</t>
         </is>
       </c>
       <c r="G92" t="inlineStr"/>
@@ -9594,7 +9594,7 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>4.3</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
@@ -9604,7 +9604,7 @@
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>1.0105</t>
+          <t>0.47</t>
         </is>
       </c>
       <c r="G99" t="inlineStr"/>
@@ -9825,7 +9825,7 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>2.2</t>
+          <t>2.8</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
@@ -9835,7 +9835,7 @@
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>0.9664</t>
+          <t>0.7593</t>
         </is>
       </c>
       <c r="G106" t="inlineStr"/>
@@ -10056,7 +10056,7 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>2.2</t>
+          <t>2.8</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
@@ -10066,7 +10066,7 @@
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>0.8599</t>
+          <t>0.6756</t>
         </is>
       </c>
       <c r="G113" t="inlineStr"/>
@@ -10122,7 +10122,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>4.1</t>
+          <t>4.3</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
@@ -10132,7 +10132,7 @@
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>0.625</t>
+          <t>0.596</t>
         </is>
       </c>
       <c r="G115" t="inlineStr"/>
@@ -10155,7 +10155,7 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>11.8</t>
+          <t>12.8</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
@@ -10165,7 +10165,7 @@
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>0.2884</t>
+          <t>0.2659</t>
         </is>
       </c>
       <c r="G116" t="inlineStr"/>

</xml_diff>